<commit_message>
feat: introduce SprintHoliday model to support holiday-aware task scheduling and standardize task status values
</commit_message>
<xml_diff>
--- a/Backend/templates/tasks_template.xlsx
+++ b/Backend/templates/tasks_template.xlsx
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Sprint Piliot AI Tasks Template</t>
   </si>
   <si>
     <t xml:space="preserve">Tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holidays</t>
   </si>
   <si>
     <t xml:space="preserve">Task Title</t>
@@ -80,10 +83,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -117,6 +121,14 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
@@ -191,28 +203,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -493,99 +521,115 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:E1002"/>
+  <dimension ref="B1:F1002"/>
   <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.97"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>5</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>46233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="5"/>
+      <c r="D5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="8"/>
+      <c r="F5" s="7" t="n">
+        <v>46234</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="5"/>
+      <c r="D6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="5"/>
+      <c r="D7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="5"/>
+      <c r="D8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1569,7 +1613,7 @@
     <row r="1002" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B1:F1"/>
     <mergeCell ref="B3:E3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>